<commit_message>
Calendrier novembre v2 (2 EVENT/mois) et budget réseaux sociaux 2027
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011boZbkbrQUBfZ2CayJHvQc
</commit_message>
<xml_diff>
--- a/livrables/calendrier-editorial-novembre-2026.xlsx
+++ b/livrables/calendrier-editorial-novembre-2026.xlsx
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P44"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -700,7 +700,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2 publications par semaine (mardi et jeudi, 12h15) · 3 piliers : PRODUITS, EVENT, TREND · Fil rouge du mois : fin d'année fiscale (versement 3a avant le 31.12)</t>
+          <t>Règle : 2 posts par semaine (mardi et jeudi, 12h15), piliers en alternance · chaque mois : 2 EVENT (1 événement L'Annexe + 1 événement partenaire), le reste en PRODUITS et TREND · Fil rouge de novembre : versement 3a avant le 31.12</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       <c r="G8" s="14" t="inlineStr">
         <is>
           <t>05.11 · EVENT · Post
-Les Midis de L'Annexe : [titre de l'atelier]</t>
+Événement L'Annexe · [titre de l'événement de novembre]</t>
         </is>
       </c>
       <c r="H8" s="15" t="n"/>
@@ -832,8 +832,8 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>17.11 · EVENT · Carrousel (4 slides)
-Soirée de L'Annexe : [thème]</t>
+          <t>17.11 · EVENT · Post collab (co-auteur)
+Événement partenaire · [nom du partenaire] × L'Annexe : [événement]</t>
         </is>
       </c>
       <c r="C10" s="15" t="n"/>
@@ -857,26 +857,26 @@
           <t>S4</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>24.11 · EVENT · Carrousel photo
-On y était : retour sur [l'atelier]</t>
-        </is>
-      </c>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="15" t="n"/>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="15" t="n"/>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>26.11 · PRODUITS · Carrousel
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>24.11 · PRODUITS · Carrousel
 31 décembre : ce qu'il faut faire avant la fin d'année pour ton 3a</t>
         </is>
       </c>
-      <c r="H11" s="13" t="n"/>
-      <c r="I11" s="13" t="n"/>
-      <c r="J11" s="13" t="n"/>
-      <c r="K11" s="13" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="13" t="n"/>
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>26.11 · TREND · Reel
+Dis-moi que tu es freelance sans me dire que tu es freelance</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="17" t="n"/>
+      <c r="J11" s="17" t="n"/>
+      <c r="K11" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -1066,12 +1066,12 @@
       </c>
       <c r="G17" s="29" t="inlineStr">
         <is>
-          <t>Les Midis de L'Annexe : [titre de l'atelier]</t>
+          <t>Événement L'Annexe · [titre de l'événement de novembre]</t>
         </is>
       </c>
       <c r="H17" s="28" t="inlineStr">
         <is>
-          <t>Date · intervenant·e · 12h-13h30 · gratuit · places limitées.</t>
+          <t>Date · intervenant·e · horaire · gratuit · places limitées. Récap en stories le jour J.</t>
         </is>
       </c>
       <c r="I17" s="28" t="inlineStr">
@@ -1086,11 +1086,11 @@
       </c>
       <c r="K17" s="28" t="inlineStr">
         <is>
-          <t>Relais + sticker « Rappel »</t>
+          <t>Relais + sticker « Rappel » + compte à rebours J-5</t>
         </is>
       </c>
       <c r="L17" s="30" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="M17" s="25" t="inlineStr">
         <is>
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="L19" s="30" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="M19" s="25" t="inlineStr">
         <is>
@@ -1268,36 +1268,36 @@
       </c>
       <c r="F20" s="22" t="inlineStr">
         <is>
-          <t>Carrousel (4 slides)</t>
+          <t>Post collab (co-auteur)</t>
         </is>
       </c>
       <c r="G20" s="23" t="inlineStr">
         <is>
-          <t>Soirée de L'Annexe : [thème]</t>
+          <t>Événement partenaire · [nom du partenaire] × L'Annexe : [événement]</t>
         </is>
       </c>
       <c r="H20" s="22" t="inlineStr">
         <is>
-          <t>Slide 1 date · 2 intervenant·e · 3 programme · 4 inscription.</t>
+          <t>Post publié en collaboration avec le partenaire (apparaît sur les 2 comptes) : date, lieu, ce qu'on y fait.</t>
         </is>
       </c>
       <c r="I20" s="22" t="inlineStr">
         <is>
-          <t>Inscris-toi, 80 places</t>
+          <t>Inscris-toi (lien du partenaire)</t>
         </is>
       </c>
       <c r="J20" s="22" t="inlineStr">
         <is>
-          <t>Post 1 (Événement)</t>
+          <t>Post 1 (Événement), logos des 2 marques</t>
         </is>
       </c>
       <c r="K20" s="22" t="inlineStr">
         <is>
-          <t>Compte à rebours J-7 à J-1</t>
+          <t>Repost des stories du partenaire</t>
         </is>
       </c>
       <c r="L20" s="24" t="n">
-        <v>800</v>
+        <v>100</v>
       </c>
       <c r="M20" s="19" t="inlineStr">
         <is>
@@ -1366,7 +1366,7 @@
         </is>
       </c>
       <c r="L21" s="30" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="M21" s="25" t="inlineStr">
         <is>
@@ -1401,41 +1401,41 @@
       </c>
       <c r="E22" s="21" t="inlineStr">
         <is>
-          <t>EVENT</t>
+          <t>PRODUITS</t>
         </is>
       </c>
       <c r="F22" s="22" t="inlineStr">
         <is>
-          <t>Carrousel photo</t>
+          <t>Carrousel</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>On y était : retour sur [l'atelier]</t>
+          <t>31 décembre : ce qu'il faut faire avant la fin d'année pour ton 3a</t>
         </is>
       </c>
       <c r="H22" s="22" t="inlineStr">
         <is>
-          <t>5 vraies photos · 3 choses à retenir · 1 citation (avec accord).</t>
+          <t>Check-list : vérifier son plafond · faire son versement · garder l'attestation.</t>
         </is>
       </c>
       <c r="I22" s="22" t="inlineStr">
         <is>
-          <t>Prochain rendez-vous le [date soirée]</t>
+          <t>Prends rendez-vous / Calcule ton économie</t>
         </is>
       </c>
       <c r="J22" s="22" t="inlineStr">
         <is>
-          <t>Post 6 (Récap) + Post 5 (Citation)</t>
+          <t>Post 2 + Post 3</t>
         </is>
       </c>
       <c r="K22" s="22" t="inlineStr">
         <is>
-          <t>Photos des coulisses</t>
+          <t>Story 1 minute prévoyance + lien</t>
         </is>
       </c>
       <c r="L22" s="24" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="M22" s="19" t="inlineStr">
         <is>
@@ -1470,41 +1470,41 @@
       </c>
       <c r="E23" s="27" t="inlineStr">
         <is>
-          <t>PRODUITS</t>
+          <t>TREND</t>
         </is>
       </c>
       <c r="F23" s="28" t="inlineStr">
         <is>
-          <t>Carrousel</t>
+          <t>Reel</t>
         </is>
       </c>
       <c r="G23" s="29" t="inlineStr">
         <is>
-          <t>31 décembre : ce qu'il faut faire avant la fin d'année pour ton 3a</t>
+          <t>Dis-moi que tu es freelance sans me dire que tu es freelance</t>
         </is>
       </c>
       <c r="H23" s="28" t="inlineStr">
         <is>
-          <t>Check-list : vérifier son plafond · faire son versement · garder l'attestation.</t>
+          <t>Format tendance : 4 situations du quotidien d'indépendant·e, la dernière : « et personne ne cotise pour ma retraite ».</t>
         </is>
       </c>
       <c r="I23" s="28" t="inlineStr">
         <is>
-          <t>Prends rendez-vous / Calcule ton économie</t>
+          <t>Dis-nous la tienne en commentaire</t>
         </is>
       </c>
       <c r="J23" s="28" t="inlineStr">
         <is>
-          <t>Post 2 + Post 3</t>
+          <t>Couverture Reel (version Photo)</t>
         </is>
       </c>
       <c r="K23" s="28" t="inlineStr">
         <is>
-          <t>Story 1 minute prévoyance + lien</t>
+          <t>Sondage « Tu as un 3a ? Oui / Pas encore »</t>
         </is>
       </c>
       <c r="L23" s="30" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="M23" s="25" t="inlineStr">
         <is>
@@ -1514,7 +1514,7 @@
       <c r="N23" s="28" t="inlineStr"/>
       <c r="O23" s="25" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Non requis</t>
         </is>
       </c>
       <c r="P23" s="28" t="inlineStr"/>
@@ -1901,7 +1901,21 @@
     <row r="44">
       <c r="A44" s="34" t="inlineStr">
         <is>
+          <t>Pub du mois : 300 (événement L'Annexe) + 100 (événement partenaire) + 300 (pub continue sur les meilleurs posts PRODUITS / TREND) + 1'500 (campagne fin d'année, couvre novembre et décembre).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="34" t="inlineStr">
+        <is>
           <t>À valider : dates et thèmes des événements [entre crochets] · contenus PRODUITS par la conformité (plafonds 3a, pas de promesse de rendement) · sons tendance à choisir la veille parmi les sons libres de droits pour compte pro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="34" t="inlineStr">
+        <is>
+          <t>Le récap de l'événement L'Annexe se fait en stories (pas de post supplémentaire), pour garder le rythme de 2 posts par semaine.</t>
         </is>
       </c>
     </row>
@@ -1957,7 +1971,7 @@
       <formula1>"PRODUITS,EVENT,TREND"</formula1>
     </dataValidation>
     <dataValidation sqref="F16:F40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Choisis une valeur dans la liste" type="list">
-      <formula1>"Reel,Carrousel,Carrousel (4 slides),Carrousel photo,Post,Story"</formula1>
+      <formula1>"Reel,Carrousel,Carrousel (4 slides),Carrousel photo,Post,Post collab (co-auteur),Story"</formula1>
     </dataValidation>
     <dataValidation sqref="M16:M40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Choisis une valeur dans la liste" type="list">
       <formula1>"À préparer,En création,En validation,Programmé,Publié"</formula1>

</xml_diff>

<commit_message>
Calendrier novembre : vue mensuelle type calendrier
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011boZbkbrQUBfZ2CayJHvQc
</commit_message>
<xml_diff>
--- a/livrables/calendrier-editorial-novembre-2026.xlsx
+++ b/livrables/calendrier-editorial-novembre-2026.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Novembre 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Calendrier" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Détail des posts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Novembre 2026'!$A$15:$P$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Détail des posts'!$A$15:$P$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,13 +19,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
     <numFmt numFmtId="166" formatCode="#,##0;-#,##0;&quot;–&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0 &quot;CHF&quot;"/>
+    <numFmt numFmtId="168" formatCode="&quot;Pub du mois : &quot;#,##0&quot; CHF&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,8 +96,44 @@
       <color rgb="00595959"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B5F86"/>
+      <sz val="26"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B5F86"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00BFBFBF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00171717"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="008C8C8C"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -127,8 +165,13 @@
         <fgColor rgb="00FAFAFA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -150,25 +193,94 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -237,7 +349,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -669,6 +780,400 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Novembre 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Calendrier éditorial Instagram · L'Annexe by RG · 2 posts par semaine (mardi et jeudi, 12h15) · 2 EVENT par mois (L'Annexe + partenaire), le reste en PRODUITS et TREND</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>PRODUITS</t>
+        </is>
+      </c>
+      <c r="B3" s="4">
+        <f>COUNTIF('Détail des posts'!$E$16:$E$40,"PRODUITS")&amp;" posts"</f>
+        <v/>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>EVENT</t>
+        </is>
+      </c>
+      <c r="D3" s="4">
+        <f>COUNTIF('Détail des posts'!$E$16:$E$40,"EVENT")&amp;" posts"</f>
+        <v/>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>TREND</t>
+        </is>
+      </c>
+      <c r="F3" s="4">
+        <f>COUNTIF('Détail des posts'!$E$16:$E$40,"TREND")&amp;" posts"</f>
+        <v/>
+      </c>
+      <c r="G3" s="7">
+        <f>'Détail des posts'!L41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" ht="96" customHeight="1">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>3   ·   PRODUITS</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>5   ·   EVENT</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" ht="96" customHeight="1">
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Carrousel (4 slides)
+Taux fixe ou taux variable ? Ton 3a expliqué en 4 slides.
+12h15</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Story · Quiz du mercredi</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Post
+Événement L'Annexe · [titre de l'événement de novembre]
+12h15  ·  pub 300 CHF</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>10   ·   TREND</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>12   ·   PRODUITS</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" ht="96" customHeight="1">
+      <c r="A11" s="15" t="n"/>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>Reel
+POV : tu découvres que ton 3a se déduit de tes impôts
+12h15</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Story · Quiz du mercredi</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Reel
+Combien tu économiserais d'impôts avec ton 3a ? On fait le test.
+12h15  ·  pub 150 CHF</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>17   ·   EVENT</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>19   ·   TREND</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" ht="96" customHeight="1">
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Post collab (co-auteur)
+Événement partenaire · [nom du partenaire] × L'Annexe : [événement]
+12h15  ·  pub 100 CHF</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Story · Quiz du mercredi</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>Reel
+Ce que j'aurais aimé savoir sur l'argent à 25 ans
+12h15  ·  pub 150 CHF</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>24   ·   PRODUITS</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>26   ·   TREND</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" ht="96" customHeight="1">
+      <c r="A15" s="15" t="n"/>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Carrousel
+31 décembre : ce qu'il faut faire avant la fin d'année pour ton 3a
+12h15  ·  pub 1'500 CHF</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>Story · Quiz du mercredi</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>Reel
+Dis-moi que tu es freelance sans me dire que tu es freelance
+12h15</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" ht="96" customHeight="1">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>Les cases colorées sont les publications (détail complet dans l'onglet « Détail des posts »). Les mercredis : story « Quiz du mercredi ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>Récap de l'événement L'Annexe en stories le jour J (pas de post en plus). Éléments [entre crochets] à compléter. Contenus PRODUITS à faire valider par la conformité.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -691,7 +1196,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Calendrier éditorial Instagram · L'Annexe by RG · Novembre 2026</t>
         </is>
@@ -705,1215 +1210,1216 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>LÉGENDE</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>PRODUITS</t>
         </is>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="24">
         <f>COUNTIF($E$16:$E$40,"PRODUITS")&amp;" posts"</f>
         <v/>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>EVENT</t>
         </is>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="24">
         <f>COUNTIF($E$16:$E$40,"EVENT")&amp;" posts"</f>
         <v/>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>TREND</t>
         </is>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="24">
         <f>COUNTIF($E$16:$E$40,"TREND")&amp;" posts"</f>
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="6" hidden="1">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>VUE DU MOIS</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="7" hidden="1">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Sem.</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="26" t="inlineStr">
         <is>
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="H7" s="10" t="n"/>
-      <c r="I7" s="10" t="n"/>
-      <c r="J7" s="10" t="n"/>
-      <c r="K7" s="10" t="n"/>
-    </row>
-    <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="H7" s="27" t="n"/>
+      <c r="I7" s="27" t="n"/>
+      <c r="J7" s="27" t="n"/>
+      <c r="K7" s="27" t="n"/>
+    </row>
+    <row r="8" hidden="1" ht="46" customHeight="1">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>03.11 · PRODUITS · Carrousel (4 slides)
 Taux fixe ou taux variable ? Ton 3a expliqué en 4 slides.</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n"/>
-      <c r="D8" s="13" t="n"/>
-      <c r="E8" s="13" t="n"/>
-      <c r="F8" s="13" t="n"/>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="C8" s="30" t="n"/>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="30" t="n"/>
+      <c r="F8" s="30" t="n"/>
+      <c r="G8" s="31" t="inlineStr">
         <is>
           <t>05.11 · EVENT · Post
 Événement L'Annexe · [titre de l'événement de novembre]</t>
         </is>
       </c>
-      <c r="H8" s="15" t="n"/>
-      <c r="I8" s="15" t="n"/>
-      <c r="J8" s="15" t="n"/>
-      <c r="K8" s="15" t="n"/>
-    </row>
-    <row r="9" ht="46" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="H8" s="32" t="n"/>
+      <c r="I8" s="32" t="n"/>
+      <c r="J8" s="32" t="n"/>
+      <c r="K8" s="32" t="n"/>
+    </row>
+    <row r="9" hidden="1" ht="46" customHeight="1">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="33" t="inlineStr">
         <is>
           <t>10.11 · TREND · Reel
 POV : tu découvres que ton 3a se déduit de tes impôts</t>
         </is>
       </c>
-      <c r="C9" s="17" t="n"/>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="17" t="n"/>
-      <c r="G9" s="12" t="inlineStr">
+      <c r="C9" s="34" t="n"/>
+      <c r="D9" s="34" t="n"/>
+      <c r="E9" s="34" t="n"/>
+      <c r="F9" s="34" t="n"/>
+      <c r="G9" s="29" t="inlineStr">
         <is>
           <t>12.11 · PRODUITS · Reel
 Combien tu économiserais d'impôts avec ton 3a ? On fait le test.</t>
         </is>
       </c>
-      <c r="H9" s="13" t="n"/>
-      <c r="I9" s="13" t="n"/>
-      <c r="J9" s="13" t="n"/>
-      <c r="K9" s="13" t="n"/>
-    </row>
-    <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="H9" s="30" t="n"/>
+      <c r="I9" s="30" t="n"/>
+      <c r="J9" s="30" t="n"/>
+      <c r="K9" s="30" t="n"/>
+    </row>
+    <row r="10" hidden="1" ht="46" customHeight="1">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="31" t="inlineStr">
         <is>
           <t>17.11 · EVENT · Post collab (co-auteur)
 Événement partenaire · [nom du partenaire] × L'Annexe : [événement]</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="16" t="inlineStr">
+      <c r="C10" s="32" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="32" t="n"/>
+      <c r="F10" s="32" t="n"/>
+      <c r="G10" s="33" t="inlineStr">
         <is>
           <t>19.11 · TREND · Reel
 Ce que j'aurais aimé savoir sur l'argent à 25 ans</t>
         </is>
       </c>
-      <c r="H10" s="17" t="n"/>
-      <c r="I10" s="17" t="n"/>
-      <c r="J10" s="17" t="n"/>
-      <c r="K10" s="17" t="n"/>
-    </row>
-    <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="H10" s="34" t="n"/>
+      <c r="I10" s="34" t="n"/>
+      <c r="J10" s="34" t="n"/>
+      <c r="K10" s="34" t="n"/>
+    </row>
+    <row r="11" hidden="1" ht="46" customHeight="1">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="29" t="inlineStr">
         <is>
           <t>24.11 · PRODUITS · Carrousel
 31 décembre : ce qu'il faut faire avant la fin d'année pour ton 3a</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="16" t="inlineStr">
+      <c r="C11" s="30" t="n"/>
+      <c r="D11" s="30" t="n"/>
+      <c r="E11" s="30" t="n"/>
+      <c r="F11" s="30" t="n"/>
+      <c r="G11" s="33" t="inlineStr">
         <is>
           <t>26.11 · TREND · Reel
 Dis-moi que tu es freelance sans me dire que tu es freelance</t>
         </is>
       </c>
-      <c r="H11" s="17" t="n"/>
-      <c r="I11" s="17" t="n"/>
-      <c r="J11" s="17" t="n"/>
-      <c r="K11" s="17" t="n"/>
-    </row>
+      <c r="H11" s="34" t="n"/>
+      <c r="I11" s="34" t="n"/>
+      <c r="J11" s="34" t="n"/>
+      <c r="K11" s="34" t="n"/>
+    </row>
+    <row r="12" hidden="1"/>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>DÉTAIL DES PUBLICATIONS</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="35" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B15" s="35" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="C15" s="35" t="inlineStr">
         <is>
           <t>Jour</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr">
+      <c r="D15" s="35" t="inlineStr">
         <is>
           <t>Semaine</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E15" s="35" t="inlineStr">
         <is>
           <t>Pilier</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F15" s="35" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
       </c>
-      <c r="G15" s="18" t="inlineStr">
+      <c r="G15" s="35" t="inlineStr">
         <is>
           <t>Titre / accroche</t>
         </is>
       </c>
-      <c r="H15" s="18" t="inlineStr">
+      <c r="H15" s="35" t="inlineStr">
         <is>
           <t>Contenu</t>
         </is>
       </c>
-      <c r="I15" s="18" t="inlineStr">
+      <c r="I15" s="35" t="inlineStr">
         <is>
           <t>Call-to-action</t>
         </is>
       </c>
-      <c r="J15" s="18" t="inlineStr">
+      <c r="J15" s="35" t="inlineStr">
         <is>
           <t>Template (canevas)</t>
         </is>
       </c>
-      <c r="K15" s="18" t="inlineStr">
+      <c r="K15" s="35" t="inlineStr">
         <is>
           <t>Story associée</t>
         </is>
       </c>
-      <c r="L15" s="18" t="inlineStr">
+      <c r="L15" s="35" t="inlineStr">
         <is>
           <t>Pub (CHF)</t>
         </is>
       </c>
-      <c r="M15" s="18" t="inlineStr">
+      <c r="M15" s="35" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="N15" s="18" t="inlineStr">
+      <c r="N15" s="35" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="O15" s="18" t="inlineStr">
+      <c r="O15" s="35" t="inlineStr">
         <is>
           <t>Conformité</t>
         </is>
       </c>
-      <c r="P15" s="18" t="inlineStr">
+      <c r="P15" s="35" t="inlineStr">
         <is>
           <t>Notes / lien visuel</t>
         </is>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="19">
+      <c r="A16" s="36">
         <f>IF(G16="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B16" s="20" t="n">
+      <c r="B16" s="37" t="n">
         <v>46329</v>
       </c>
-      <c r="C16" s="19" t="inlineStr">
+      <c r="C16" s="36" t="inlineStr">
         <is>
           <t>Mardi</t>
         </is>
       </c>
-      <c r="D16" s="19" t="inlineStr">
+      <c r="D16" s="36" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="E16" s="21" t="inlineStr">
+      <c r="E16" s="38" t="inlineStr">
         <is>
           <t>PRODUITS</t>
         </is>
       </c>
-      <c r="F16" s="22" t="inlineStr">
+      <c r="F16" s="39" t="inlineStr">
         <is>
           <t>Carrousel (4 slides)</t>
         </is>
       </c>
-      <c r="G16" s="23" t="inlineStr">
+      <c r="G16" s="40" t="inlineStr">
         <is>
           <t>Taux fixe ou taux variable ? Ton 3a expliqué en 4 slides.</t>
         </is>
       </c>
-      <c r="H16" s="22" t="inlineStr">
+      <c r="H16" s="39" t="inlineStr">
         <is>
           <t>Les 2 options du 3e pilier A · pour qui chacune · capital ou rente à vie.</t>
         </is>
       </c>
-      <c r="I16" s="22" t="inlineStr">
+      <c r="I16" s="39" t="inlineStr">
         <is>
           <t>Enregistre ce post pour plus tard</t>
         </is>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="39" t="inlineStr">
         <is>
           <t>Post 2 (couverture) + Post 3 (slides)</t>
         </is>
       </c>
-      <c r="K16" s="22" t="inlineStr">
+      <c r="K16" s="39" t="inlineStr">
         <is>
           <t>Relais du post + sondage « Tu connaissais ? »</t>
         </is>
       </c>
-      <c r="L16" s="24" t="n">
+      <c r="L16" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="M16" s="19" t="inlineStr">
+      <c r="M16" s="36" t="inlineStr">
         <is>
           <t>À préparer</t>
         </is>
       </c>
-      <c r="N16" s="22" t="inlineStr"/>
-      <c r="O16" s="19" t="inlineStr">
+      <c r="N16" s="39" t="inlineStr"/>
+      <c r="O16" s="36" t="inlineStr">
         <is>
           <t>À faire</t>
         </is>
       </c>
-      <c r="P16" s="22" t="inlineStr"/>
+      <c r="P16" s="39" t="inlineStr"/>
     </row>
     <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="25">
+      <c r="A17" s="42">
         <f>IF(G17="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B17" s="26" t="n">
+      <c r="B17" s="43" t="n">
         <v>46331</v>
       </c>
-      <c r="C17" s="25" t="inlineStr">
+      <c r="C17" s="42" t="inlineStr">
         <is>
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="D17" s="25" t="inlineStr">
+      <c r="D17" s="42" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="E17" s="27" t="inlineStr">
+      <c r="E17" s="44" t="inlineStr">
         <is>
           <t>EVENT</t>
         </is>
       </c>
-      <c r="F17" s="28" t="inlineStr">
+      <c r="F17" s="45" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="G17" s="29" t="inlineStr">
+      <c r="G17" s="46" t="inlineStr">
         <is>
           <t>Événement L'Annexe · [titre de l'événement de novembre]</t>
         </is>
       </c>
-      <c r="H17" s="28" t="inlineStr">
+      <c r="H17" s="45" t="inlineStr">
         <is>
           <t>Date · intervenant·e · horaire · gratuit · places limitées. Récap en stories le jour J.</t>
         </is>
       </c>
-      <c r="I17" s="28" t="inlineStr">
+      <c r="I17" s="45" t="inlineStr">
         <is>
           <t>Réserve ta place (lien en bio)</t>
         </is>
       </c>
-      <c r="J17" s="28" t="inlineStr">
+      <c r="J17" s="45" t="inlineStr">
         <is>
           <t>Post 1 (Événement)</t>
         </is>
       </c>
-      <c r="K17" s="28" t="inlineStr">
+      <c r="K17" s="45" t="inlineStr">
         <is>
           <t>Relais + sticker « Rappel » + compte à rebours J-5</t>
         </is>
       </c>
-      <c r="L17" s="30" t="n">
+      <c r="L17" s="47" t="n">
         <v>300</v>
       </c>
-      <c r="M17" s="25" t="inlineStr">
+      <c r="M17" s="42" t="inlineStr">
         <is>
           <t>À préparer</t>
         </is>
       </c>
-      <c r="N17" s="28" t="inlineStr"/>
-      <c r="O17" s="25" t="inlineStr">
+      <c r="N17" s="45" t="inlineStr"/>
+      <c r="O17" s="42" t="inlineStr">
         <is>
           <t>À faire</t>
         </is>
       </c>
-      <c r="P17" s="28" t="inlineStr"/>
+      <c r="P17" s="45" t="inlineStr"/>
     </row>
     <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="19">
+      <c r="A18" s="36">
         <f>IF(G18="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B18" s="20" t="n">
+      <c r="B18" s="37" t="n">
         <v>46336</v>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="C18" s="36" t="inlineStr">
         <is>
           <t>Mardi</t>
         </is>
       </c>
-      <c r="D18" s="19" t="inlineStr">
+      <c r="D18" s="36" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="E18" s="21" t="inlineStr">
+      <c r="E18" s="38" t="inlineStr">
         <is>
           <t>TREND</t>
         </is>
       </c>
-      <c r="F18" s="22" t="inlineStr">
+      <c r="F18" s="39" t="inlineStr">
         <is>
           <t>Reel</t>
         </is>
       </c>
-      <c r="G18" s="23" t="inlineStr">
+      <c r="G18" s="40" t="inlineStr">
         <is>
           <t>POV : tu découvres que ton 3a se déduit de tes impôts</t>
         </is>
       </c>
-      <c r="H18" s="22" t="inlineStr">
+      <c r="H18" s="39" t="inlineStr">
         <is>
           <t>Réaction filmée à L'Annexe sur un son tendance du moment.</t>
         </is>
       </c>
-      <c r="I18" s="22" t="inlineStr">
+      <c r="I18" s="39" t="inlineStr">
         <is>
           <t>Tague la personne qui ne le sait pas encore</t>
         </is>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="39" t="inlineStr">
         <is>
           <t>Couverture Reel (version Photo)</t>
         </is>
       </c>
-      <c r="K18" s="22" t="inlineStr">
+      <c r="K18" s="39" t="inlineStr">
         <is>
           <t>Repost du Reel</t>
         </is>
       </c>
-      <c r="L18" s="24" t="n">
+      <c r="L18" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="M18" s="19" t="inlineStr">
+      <c r="M18" s="36" t="inlineStr">
         <is>
           <t>À préparer</t>
         </is>
       </c>
-      <c r="N18" s="22" t="inlineStr"/>
-      <c r="O18" s="19" t="inlineStr">
+      <c r="N18" s="39" t="inlineStr"/>
+      <c r="O18" s="36" t="inlineStr">
         <is>
           <t>Non requis</t>
         </is>
       </c>
-      <c r="P18" s="22" t="inlineStr"/>
+      <c r="P18" s="39" t="inlineStr"/>
     </row>
     <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="25">
+      <c r="A19" s="42">
         <f>IF(G19="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B19" s="26" t="n">
+      <c r="B19" s="43" t="n">
         <v>46338</v>
       </c>
-      <c r="C19" s="25" t="inlineStr">
+      <c r="C19" s="42" t="inlineStr">
         <is>
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="D19" s="25" t="inlineStr">
+      <c r="D19" s="42" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="E19" s="27" t="inlineStr">
+      <c r="E19" s="44" t="inlineStr">
         <is>
           <t>PRODUITS</t>
         </is>
       </c>
-      <c r="F19" s="28" t="inlineStr">
+      <c r="F19" s="45" t="inlineStr">
         <is>
           <t>Reel</t>
         </is>
       </c>
-      <c r="G19" s="29" t="inlineStr">
+      <c r="G19" s="46" t="inlineStr">
         <is>
           <t>Combien tu économiserais d'impôts avec ton 3a ? On fait le test.</t>
         </is>
       </c>
-      <c r="H19" s="28" t="inlineStr">
+      <c r="H19" s="45" t="inlineStr">
         <is>
           <t>Une personne de l'équipe remplit le simulateur à l'écran (sans montant personnel).</t>
         </is>
       </c>
-      <c r="I19" s="28" t="inlineStr">
+      <c r="I19" s="45" t="inlineStr">
         <is>
           <t>Fais le test (lien en bio)</t>
         </is>
       </c>
-      <c r="J19" s="28" t="inlineStr">
+      <c r="J19" s="45" t="inlineStr">
         <is>
           <t>Couverture Reel (Prévoyance)</t>
         </is>
       </c>
-      <c r="K19" s="28" t="inlineStr">
+      <c r="K19" s="45" t="inlineStr">
         <is>
           <t>Conversation Léa &amp; Sam + lien simulateur</t>
         </is>
       </c>
-      <c r="L19" s="30" t="n">
+      <c r="L19" s="47" t="n">
         <v>150</v>
       </c>
-      <c r="M19" s="25" t="inlineStr">
+      <c r="M19" s="42" t="inlineStr">
         <is>
           <t>À préparer</t>
         </is>
       </c>
-      <c r="N19" s="28" t="inlineStr"/>
-      <c r="O19" s="25" t="inlineStr">
+      <c r="N19" s="45" t="inlineStr"/>
+      <c r="O19" s="42" t="inlineStr">
         <is>
           <t>À faire</t>
         </is>
       </c>
-      <c r="P19" s="28" t="inlineStr"/>
+      <c r="P19" s="45" t="inlineStr"/>
     </row>
     <row r="20" ht="42" customHeight="1">
-      <c r="A20" s="19">
+      <c r="A20" s="36">
         <f>IF(G20="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B20" s="20" t="n">
+      <c r="B20" s="37" t="n">
         <v>46343</v>
       </c>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="C20" s="36" t="inlineStr">
         <is>
           <t>Mardi</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D20" s="36" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="E20" s="21" t="inlineStr">
+      <c r="E20" s="38" t="inlineStr">
         <is>
           <t>EVENT</t>
         </is>
       </c>
-      <c r="F20" s="22" t="inlineStr">
+      <c r="F20" s="39" t="inlineStr">
         <is>
           <t>Post collab (co-auteur)</t>
         </is>
       </c>
-      <c r="G20" s="23" t="inlineStr">
+      <c r="G20" s="40" t="inlineStr">
         <is>
           <t>Événement partenaire · [nom du partenaire] × L'Annexe : [événement]</t>
         </is>
       </c>
-      <c r="H20" s="22" t="inlineStr">
+      <c r="H20" s="39" t="inlineStr">
         <is>
           <t>Post publié en collaboration avec le partenaire (apparaît sur les 2 comptes) : date, lieu, ce qu'on y fait.</t>
         </is>
       </c>
-      <c r="I20" s="22" t="inlineStr">
+      <c r="I20" s="39" t="inlineStr">
         <is>
           <t>Inscris-toi (lien du partenaire)</t>
         </is>
       </c>
-      <c r="J20" s="22" t="inlineStr">
+      <c r="J20" s="39" t="inlineStr">
         <is>
           <t>Post 1 (Événement), logos des 2 marques</t>
         </is>
       </c>
-      <c r="K20" s="22" t="inlineStr">
+      <c r="K20" s="39" t="inlineStr">
         <is>
           <t>Repost des stories du partenaire</t>
         </is>
       </c>
-      <c r="L20" s="24" t="n">
+      <c r="L20" s="41" t="n">
         <v>100</v>
       </c>
-      <c r="M20" s="19" t="inlineStr">
+      <c r="M20" s="36" t="inlineStr">
         <is>
           <t>À préparer</t>
         </is>
       </c>
-      <c r="N20" s="22" t="inlineStr"/>
-      <c r="O20" s="19" t="inlineStr">
+      <c r="N20" s="39" t="inlineStr"/>
+      <c r="O20" s="36" t="inlineStr">
         <is>
           <t>À faire</t>
         </is>
       </c>
-      <c r="P20" s="22" t="inlineStr"/>
+      <c r="P20" s="39" t="inlineStr"/>
     </row>
     <row r="21" ht="42" customHeight="1">
-      <c r="A21" s="25">
+      <c r="A21" s="42">
         <f>IF(G21="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B21" s="26" t="n">
+      <c r="B21" s="43" t="n">
         <v>46345</v>
       </c>
-      <c r="C21" s="25" t="inlineStr">
+      <c r="C21" s="42" t="inlineStr">
         <is>
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="D21" s="25" t="inlineStr">
+      <c r="D21" s="42" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="E21" s="27" t="inlineStr">
+      <c r="E21" s="44" t="inlineStr">
         <is>
           <t>TREND</t>
         </is>
       </c>
-      <c r="F21" s="28" t="inlineStr">
+      <c r="F21" s="45" t="inlineStr">
         <is>
           <t>Reel</t>
         </is>
       </c>
-      <c r="G21" s="29" t="inlineStr">
+      <c r="G21" s="46" t="inlineStr">
         <is>
           <t>Ce que j'aurais aimé savoir sur l'argent à 25 ans</t>
         </is>
       </c>
-      <c r="H21" s="28" t="inlineStr">
+      <c r="H21" s="45" t="inlineStr">
         <is>
           <t>3 jeunes de la communauté ou de l'équipe, 1 phrase chacun.</t>
         </is>
       </c>
-      <c r="I21" s="28" t="inlineStr">
+      <c r="I21" s="45" t="inlineStr">
         <is>
           <t>Et toi, tu dirais quoi ? En commentaire</t>
         </is>
       </c>
-      <c r="J21" s="28" t="inlineStr">
+      <c r="J21" s="45" t="inlineStr">
         <is>
           <t>Couverture Reel (version Photo)</t>
         </is>
       </c>
-      <c r="K21" s="28" t="inlineStr">
+      <c r="K21" s="45" t="inlineStr">
         <is>
           <t>Boîte à questions sur le thème</t>
         </is>
       </c>
-      <c r="L21" s="30" t="n">
+      <c r="L21" s="47" t="n">
         <v>150</v>
       </c>
-      <c r="M21" s="25" t="inlineStr">
+      <c r="M21" s="42" t="inlineStr">
         <is>
           <t>À préparer</t>
         </is>
       </c>
-      <c r="N21" s="28" t="inlineStr"/>
-      <c r="O21" s="25" t="inlineStr">
+      <c r="N21" s="45" t="inlineStr"/>
+      <c r="O21" s="42" t="inlineStr">
         <is>
           <t>Non requis</t>
         </is>
       </c>
-      <c r="P21" s="28" t="inlineStr"/>
+      <c r="P21" s="45" t="inlineStr"/>
     </row>
     <row r="22" ht="42" customHeight="1">
-      <c r="A22" s="19">
+      <c r="A22" s="36">
         <f>IF(G22="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B22" s="20" t="n">
+      <c r="B22" s="37" t="n">
         <v>46350</v>
       </c>
-      <c r="C22" s="19" t="inlineStr">
+      <c r="C22" s="36" t="inlineStr">
         <is>
           <t>Mardi</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
+      <c r="D22" s="36" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="E22" s="21" t="inlineStr">
+      <c r="E22" s="38" t="inlineStr">
         <is>
           <t>PRODUITS</t>
         </is>
       </c>
-      <c r="F22" s="22" t="inlineStr">
+      <c r="F22" s="39" t="inlineStr">
         <is>
           <t>Carrousel</t>
         </is>
       </c>
-      <c r="G22" s="23" t="inlineStr">
+      <c r="G22" s="40" t="inlineStr">
         <is>
           <t>31 décembre : ce qu'il faut faire avant la fin d'année pour ton 3a</t>
         </is>
       </c>
-      <c r="H22" s="22" t="inlineStr">
+      <c r="H22" s="39" t="inlineStr">
         <is>
           <t>Check-list : vérifier son plafond · faire son versement · garder l'attestation.</t>
         </is>
       </c>
-      <c r="I22" s="22" t="inlineStr">
+      <c r="I22" s="39" t="inlineStr">
         <is>
           <t>Prends rendez-vous / Calcule ton économie</t>
         </is>
       </c>
-      <c r="J22" s="22" t="inlineStr">
+      <c r="J22" s="39" t="inlineStr">
         <is>
           <t>Post 2 + Post 3</t>
         </is>
       </c>
-      <c r="K22" s="22" t="inlineStr">
+      <c r="K22" s="39" t="inlineStr">
         <is>
           <t>Story 1 minute prévoyance + lien</t>
         </is>
       </c>
-      <c r="L22" s="24" t="n">
+      <c r="L22" s="41" t="n">
         <v>1500</v>
       </c>
-      <c r="M22" s="19" t="inlineStr">
+      <c r="M22" s="36" t="inlineStr">
         <is>
           <t>À préparer</t>
         </is>
       </c>
-      <c r="N22" s="22" t="inlineStr"/>
-      <c r="O22" s="19" t="inlineStr">
+      <c r="N22" s="39" t="inlineStr"/>
+      <c r="O22" s="36" t="inlineStr">
         <is>
           <t>À faire</t>
         </is>
       </c>
-      <c r="P22" s="22" t="inlineStr"/>
+      <c r="P22" s="39" t="inlineStr"/>
     </row>
     <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="25">
+      <c r="A23" s="42">
         <f>IF(G23="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B23" s="26" t="n">
+      <c r="B23" s="43" t="n">
         <v>46352</v>
       </c>
-      <c r="C23" s="25" t="inlineStr">
+      <c r="C23" s="42" t="inlineStr">
         <is>
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="D23" s="25" t="inlineStr">
+      <c r="D23" s="42" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="E23" s="27" t="inlineStr">
+      <c r="E23" s="44" t="inlineStr">
         <is>
           <t>TREND</t>
         </is>
       </c>
-      <c r="F23" s="28" t="inlineStr">
+      <c r="F23" s="45" t="inlineStr">
         <is>
           <t>Reel</t>
         </is>
       </c>
-      <c r="G23" s="29" t="inlineStr">
+      <c r="G23" s="46" t="inlineStr">
         <is>
           <t>Dis-moi que tu es freelance sans me dire que tu es freelance</t>
         </is>
       </c>
-      <c r="H23" s="28" t="inlineStr">
+      <c r="H23" s="45" t="inlineStr">
         <is>
           <t>Format tendance : 4 situations du quotidien d'indépendant·e, la dernière : « et personne ne cotise pour ma retraite ».</t>
         </is>
       </c>
-      <c r="I23" s="28" t="inlineStr">
+      <c r="I23" s="45" t="inlineStr">
         <is>
           <t>Dis-nous la tienne en commentaire</t>
         </is>
       </c>
-      <c r="J23" s="28" t="inlineStr">
+      <c r="J23" s="45" t="inlineStr">
         <is>
           <t>Couverture Reel (version Photo)</t>
         </is>
       </c>
-      <c r="K23" s="28" t="inlineStr">
+      <c r="K23" s="45" t="inlineStr">
         <is>
           <t>Sondage « Tu as un 3a ? Oui / Pas encore »</t>
         </is>
       </c>
-      <c r="L23" s="30" t="n">
+      <c r="L23" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="M23" s="25" t="inlineStr">
+      <c r="M23" s="42" t="inlineStr">
         <is>
           <t>À préparer</t>
         </is>
       </c>
-      <c r="N23" s="28" t="inlineStr"/>
-      <c r="O23" s="25" t="inlineStr">
+      <c r="N23" s="45" t="inlineStr"/>
+      <c r="O23" s="42" t="inlineStr">
         <is>
           <t>Non requis</t>
         </is>
       </c>
-      <c r="P23" s="28" t="inlineStr"/>
+      <c r="P23" s="45" t="inlineStr"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="19">
+      <c r="A24" s="36">
         <f>IF(G24="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B24" s="20" t="n"/>
-      <c r="C24" s="19" t="n"/>
-      <c r="D24" s="19" t="n"/>
-      <c r="E24" s="21" t="n"/>
-      <c r="F24" s="22" t="n"/>
-      <c r="G24" s="23" t="n"/>
-      <c r="H24" s="22" t="n"/>
-      <c r="I24" s="22" t="n"/>
-      <c r="J24" s="22" t="n"/>
-      <c r="K24" s="22" t="n"/>
-      <c r="L24" s="24" t="n"/>
-      <c r="M24" s="19" t="n"/>
-      <c r="N24" s="22" t="n"/>
-      <c r="O24" s="19" t="n"/>
-      <c r="P24" s="22" t="n"/>
+      <c r="B24" s="37" t="n"/>
+      <c r="C24" s="36" t="n"/>
+      <c r="D24" s="36" t="n"/>
+      <c r="E24" s="38" t="n"/>
+      <c r="F24" s="39" t="n"/>
+      <c r="G24" s="40" t="n"/>
+      <c r="H24" s="39" t="n"/>
+      <c r="I24" s="39" t="n"/>
+      <c r="J24" s="39" t="n"/>
+      <c r="K24" s="39" t="n"/>
+      <c r="L24" s="41" t="n"/>
+      <c r="M24" s="36" t="n"/>
+      <c r="N24" s="39" t="n"/>
+      <c r="O24" s="36" t="n"/>
+      <c r="P24" s="39" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="25">
+      <c r="A25" s="42">
         <f>IF(G25="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B25" s="26" t="n"/>
-      <c r="C25" s="25" t="n"/>
-      <c r="D25" s="25" t="n"/>
-      <c r="E25" s="27" t="n"/>
-      <c r="F25" s="28" t="n"/>
-      <c r="G25" s="29" t="n"/>
-      <c r="H25" s="28" t="n"/>
-      <c r="I25" s="28" t="n"/>
-      <c r="J25" s="28" t="n"/>
-      <c r="K25" s="28" t="n"/>
-      <c r="L25" s="30" t="n"/>
-      <c r="M25" s="25" t="n"/>
-      <c r="N25" s="28" t="n"/>
-      <c r="O25" s="25" t="n"/>
-      <c r="P25" s="28" t="n"/>
+      <c r="B25" s="43" t="n"/>
+      <c r="C25" s="42" t="n"/>
+      <c r="D25" s="42" t="n"/>
+      <c r="E25" s="44" t="n"/>
+      <c r="F25" s="45" t="n"/>
+      <c r="G25" s="46" t="n"/>
+      <c r="H25" s="45" t="n"/>
+      <c r="I25" s="45" t="n"/>
+      <c r="J25" s="45" t="n"/>
+      <c r="K25" s="45" t="n"/>
+      <c r="L25" s="47" t="n"/>
+      <c r="M25" s="42" t="n"/>
+      <c r="N25" s="45" t="n"/>
+      <c r="O25" s="42" t="n"/>
+      <c r="P25" s="45" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="19">
+      <c r="A26" s="36">
         <f>IF(G26="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B26" s="20" t="n"/>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="19" t="n"/>
-      <c r="E26" s="21" t="n"/>
-      <c r="F26" s="22" t="n"/>
-      <c r="G26" s="23" t="n"/>
-      <c r="H26" s="22" t="n"/>
-      <c r="I26" s="22" t="n"/>
-      <c r="J26" s="22" t="n"/>
-      <c r="K26" s="22" t="n"/>
-      <c r="L26" s="24" t="n"/>
-      <c r="M26" s="19" t="n"/>
-      <c r="N26" s="22" t="n"/>
-      <c r="O26" s="19" t="n"/>
-      <c r="P26" s="22" t="n"/>
+      <c r="B26" s="37" t="n"/>
+      <c r="C26" s="36" t="n"/>
+      <c r="D26" s="36" t="n"/>
+      <c r="E26" s="38" t="n"/>
+      <c r="F26" s="39" t="n"/>
+      <c r="G26" s="40" t="n"/>
+      <c r="H26" s="39" t="n"/>
+      <c r="I26" s="39" t="n"/>
+      <c r="J26" s="39" t="n"/>
+      <c r="K26" s="39" t="n"/>
+      <c r="L26" s="41" t="n"/>
+      <c r="M26" s="36" t="n"/>
+      <c r="N26" s="39" t="n"/>
+      <c r="O26" s="36" t="n"/>
+      <c r="P26" s="39" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="25">
+      <c r="A27" s="42">
         <f>IF(G27="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B27" s="26" t="n"/>
-      <c r="C27" s="25" t="n"/>
-      <c r="D27" s="25" t="n"/>
-      <c r="E27" s="27" t="n"/>
-      <c r="F27" s="28" t="n"/>
-      <c r="G27" s="29" t="n"/>
-      <c r="H27" s="28" t="n"/>
-      <c r="I27" s="28" t="n"/>
-      <c r="J27" s="28" t="n"/>
-      <c r="K27" s="28" t="n"/>
-      <c r="L27" s="30" t="n"/>
-      <c r="M27" s="25" t="n"/>
-      <c r="N27" s="28" t="n"/>
-      <c r="O27" s="25" t="n"/>
-      <c r="P27" s="28" t="n"/>
+      <c r="B27" s="43" t="n"/>
+      <c r="C27" s="42" t="n"/>
+      <c r="D27" s="42" t="n"/>
+      <c r="E27" s="44" t="n"/>
+      <c r="F27" s="45" t="n"/>
+      <c r="G27" s="46" t="n"/>
+      <c r="H27" s="45" t="n"/>
+      <c r="I27" s="45" t="n"/>
+      <c r="J27" s="45" t="n"/>
+      <c r="K27" s="45" t="n"/>
+      <c r="L27" s="47" t="n"/>
+      <c r="M27" s="42" t="n"/>
+      <c r="N27" s="45" t="n"/>
+      <c r="O27" s="42" t="n"/>
+      <c r="P27" s="45" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="19">
+      <c r="A28" s="36">
         <f>IF(G28="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B28" s="20" t="n"/>
-      <c r="C28" s="19" t="n"/>
-      <c r="D28" s="19" t="n"/>
-      <c r="E28" s="21" t="n"/>
-      <c r="F28" s="22" t="n"/>
-      <c r="G28" s="23" t="n"/>
-      <c r="H28" s="22" t="n"/>
-      <c r="I28" s="22" t="n"/>
-      <c r="J28" s="22" t="n"/>
-      <c r="K28" s="22" t="n"/>
-      <c r="L28" s="24" t="n"/>
-      <c r="M28" s="19" t="n"/>
-      <c r="N28" s="22" t="n"/>
-      <c r="O28" s="19" t="n"/>
-      <c r="P28" s="22" t="n"/>
+      <c r="B28" s="37" t="n"/>
+      <c r="C28" s="36" t="n"/>
+      <c r="D28" s="36" t="n"/>
+      <c r="E28" s="38" t="n"/>
+      <c r="F28" s="39" t="n"/>
+      <c r="G28" s="40" t="n"/>
+      <c r="H28" s="39" t="n"/>
+      <c r="I28" s="39" t="n"/>
+      <c r="J28" s="39" t="n"/>
+      <c r="K28" s="39" t="n"/>
+      <c r="L28" s="41" t="n"/>
+      <c r="M28" s="36" t="n"/>
+      <c r="N28" s="39" t="n"/>
+      <c r="O28" s="36" t="n"/>
+      <c r="P28" s="39" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="25">
+      <c r="A29" s="42">
         <f>IF(G29="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B29" s="26" t="n"/>
-      <c r="C29" s="25" t="n"/>
-      <c r="D29" s="25" t="n"/>
-      <c r="E29" s="27" t="n"/>
-      <c r="F29" s="28" t="n"/>
-      <c r="G29" s="29" t="n"/>
-      <c r="H29" s="28" t="n"/>
-      <c r="I29" s="28" t="n"/>
-      <c r="J29" s="28" t="n"/>
-      <c r="K29" s="28" t="n"/>
-      <c r="L29" s="30" t="n"/>
-      <c r="M29" s="25" t="n"/>
-      <c r="N29" s="28" t="n"/>
-      <c r="O29" s="25" t="n"/>
-      <c r="P29" s="28" t="n"/>
+      <c r="B29" s="43" t="n"/>
+      <c r="C29" s="42" t="n"/>
+      <c r="D29" s="42" t="n"/>
+      <c r="E29" s="44" t="n"/>
+      <c r="F29" s="45" t="n"/>
+      <c r="G29" s="46" t="n"/>
+      <c r="H29" s="45" t="n"/>
+      <c r="I29" s="45" t="n"/>
+      <c r="J29" s="45" t="n"/>
+      <c r="K29" s="45" t="n"/>
+      <c r="L29" s="47" t="n"/>
+      <c r="M29" s="42" t="n"/>
+      <c r="N29" s="45" t="n"/>
+      <c r="O29" s="42" t="n"/>
+      <c r="P29" s="45" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="19">
+      <c r="A30" s="36">
         <f>IF(G30="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B30" s="20" t="n"/>
-      <c r="C30" s="19" t="n"/>
-      <c r="D30" s="19" t="n"/>
-      <c r="E30" s="21" t="n"/>
-      <c r="F30" s="22" t="n"/>
-      <c r="G30" s="23" t="n"/>
-      <c r="H30" s="22" t="n"/>
-      <c r="I30" s="22" t="n"/>
-      <c r="J30" s="22" t="n"/>
-      <c r="K30" s="22" t="n"/>
-      <c r="L30" s="24" t="n"/>
-      <c r="M30" s="19" t="n"/>
-      <c r="N30" s="22" t="n"/>
-      <c r="O30" s="19" t="n"/>
-      <c r="P30" s="22" t="n"/>
+      <c r="B30" s="37" t="n"/>
+      <c r="C30" s="36" t="n"/>
+      <c r="D30" s="36" t="n"/>
+      <c r="E30" s="38" t="n"/>
+      <c r="F30" s="39" t="n"/>
+      <c r="G30" s="40" t="n"/>
+      <c r="H30" s="39" t="n"/>
+      <c r="I30" s="39" t="n"/>
+      <c r="J30" s="39" t="n"/>
+      <c r="K30" s="39" t="n"/>
+      <c r="L30" s="41" t="n"/>
+      <c r="M30" s="36" t="n"/>
+      <c r="N30" s="39" t="n"/>
+      <c r="O30" s="36" t="n"/>
+      <c r="P30" s="39" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="25">
+      <c r="A31" s="42">
         <f>IF(G31="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B31" s="26" t="n"/>
-      <c r="C31" s="25" t="n"/>
-      <c r="D31" s="25" t="n"/>
-      <c r="E31" s="27" t="n"/>
-      <c r="F31" s="28" t="n"/>
-      <c r="G31" s="29" t="n"/>
-      <c r="H31" s="28" t="n"/>
-      <c r="I31" s="28" t="n"/>
-      <c r="J31" s="28" t="n"/>
-      <c r="K31" s="28" t="n"/>
-      <c r="L31" s="30" t="n"/>
-      <c r="M31" s="25" t="n"/>
-      <c r="N31" s="28" t="n"/>
-      <c r="O31" s="25" t="n"/>
-      <c r="P31" s="28" t="n"/>
+      <c r="B31" s="43" t="n"/>
+      <c r="C31" s="42" t="n"/>
+      <c r="D31" s="42" t="n"/>
+      <c r="E31" s="44" t="n"/>
+      <c r="F31" s="45" t="n"/>
+      <c r="G31" s="46" t="n"/>
+      <c r="H31" s="45" t="n"/>
+      <c r="I31" s="45" t="n"/>
+      <c r="J31" s="45" t="n"/>
+      <c r="K31" s="45" t="n"/>
+      <c r="L31" s="47" t="n"/>
+      <c r="M31" s="42" t="n"/>
+      <c r="N31" s="45" t="n"/>
+      <c r="O31" s="42" t="n"/>
+      <c r="P31" s="45" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="19">
+      <c r="A32" s="36">
         <f>IF(G32="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B32" s="20" t="n"/>
-      <c r="C32" s="19" t="n"/>
-      <c r="D32" s="19" t="n"/>
-      <c r="E32" s="21" t="n"/>
-      <c r="F32" s="22" t="n"/>
-      <c r="G32" s="23" t="n"/>
-      <c r="H32" s="22" t="n"/>
-      <c r="I32" s="22" t="n"/>
-      <c r="J32" s="22" t="n"/>
-      <c r="K32" s="22" t="n"/>
-      <c r="L32" s="24" t="n"/>
-      <c r="M32" s="19" t="n"/>
-      <c r="N32" s="22" t="n"/>
-      <c r="O32" s="19" t="n"/>
-      <c r="P32" s="22" t="n"/>
+      <c r="B32" s="37" t="n"/>
+      <c r="C32" s="36" t="n"/>
+      <c r="D32" s="36" t="n"/>
+      <c r="E32" s="38" t="n"/>
+      <c r="F32" s="39" t="n"/>
+      <c r="G32" s="40" t="n"/>
+      <c r="H32" s="39" t="n"/>
+      <c r="I32" s="39" t="n"/>
+      <c r="J32" s="39" t="n"/>
+      <c r="K32" s="39" t="n"/>
+      <c r="L32" s="41" t="n"/>
+      <c r="M32" s="36" t="n"/>
+      <c r="N32" s="39" t="n"/>
+      <c r="O32" s="36" t="n"/>
+      <c r="P32" s="39" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="25">
+      <c r="A33" s="42">
         <f>IF(G33="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B33" s="26" t="n"/>
-      <c r="C33" s="25" t="n"/>
-      <c r="D33" s="25" t="n"/>
-      <c r="E33" s="27" t="n"/>
-      <c r="F33" s="28" t="n"/>
-      <c r="G33" s="29" t="n"/>
-      <c r="H33" s="28" t="n"/>
-      <c r="I33" s="28" t="n"/>
-      <c r="J33" s="28" t="n"/>
-      <c r="K33" s="28" t="n"/>
-      <c r="L33" s="30" t="n"/>
-      <c r="M33" s="25" t="n"/>
-      <c r="N33" s="28" t="n"/>
-      <c r="O33" s="25" t="n"/>
-      <c r="P33" s="28" t="n"/>
+      <c r="B33" s="43" t="n"/>
+      <c r="C33" s="42" t="n"/>
+      <c r="D33" s="42" t="n"/>
+      <c r="E33" s="44" t="n"/>
+      <c r="F33" s="45" t="n"/>
+      <c r="G33" s="46" t="n"/>
+      <c r="H33" s="45" t="n"/>
+      <c r="I33" s="45" t="n"/>
+      <c r="J33" s="45" t="n"/>
+      <c r="K33" s="45" t="n"/>
+      <c r="L33" s="47" t="n"/>
+      <c r="M33" s="42" t="n"/>
+      <c r="N33" s="45" t="n"/>
+      <c r="O33" s="42" t="n"/>
+      <c r="P33" s="45" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="19">
+      <c r="A34" s="36">
         <f>IF(G34="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B34" s="20" t="n"/>
-      <c r="C34" s="19" t="n"/>
-      <c r="D34" s="19" t="n"/>
-      <c r="E34" s="21" t="n"/>
-      <c r="F34" s="22" t="n"/>
-      <c r="G34" s="23" t="n"/>
-      <c r="H34" s="22" t="n"/>
-      <c r="I34" s="22" t="n"/>
-      <c r="J34" s="22" t="n"/>
-      <c r="K34" s="22" t="n"/>
-      <c r="L34" s="24" t="n"/>
-      <c r="M34" s="19" t="n"/>
-      <c r="N34" s="22" t="n"/>
-      <c r="O34" s="19" t="n"/>
-      <c r="P34" s="22" t="n"/>
+      <c r="B34" s="37" t="n"/>
+      <c r="C34" s="36" t="n"/>
+      <c r="D34" s="36" t="n"/>
+      <c r="E34" s="38" t="n"/>
+      <c r="F34" s="39" t="n"/>
+      <c r="G34" s="40" t="n"/>
+      <c r="H34" s="39" t="n"/>
+      <c r="I34" s="39" t="n"/>
+      <c r="J34" s="39" t="n"/>
+      <c r="K34" s="39" t="n"/>
+      <c r="L34" s="41" t="n"/>
+      <c r="M34" s="36" t="n"/>
+      <c r="N34" s="39" t="n"/>
+      <c r="O34" s="36" t="n"/>
+      <c r="P34" s="39" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="25">
+      <c r="A35" s="42">
         <f>IF(G35="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B35" s="26" t="n"/>
-      <c r="C35" s="25" t="n"/>
-      <c r="D35" s="25" t="n"/>
-      <c r="E35" s="27" t="n"/>
-      <c r="F35" s="28" t="n"/>
-      <c r="G35" s="29" t="n"/>
-      <c r="H35" s="28" t="n"/>
-      <c r="I35" s="28" t="n"/>
-      <c r="J35" s="28" t="n"/>
-      <c r="K35" s="28" t="n"/>
-      <c r="L35" s="30" t="n"/>
-      <c r="M35" s="25" t="n"/>
-      <c r="N35" s="28" t="n"/>
-      <c r="O35" s="25" t="n"/>
-      <c r="P35" s="28" t="n"/>
+      <c r="B35" s="43" t="n"/>
+      <c r="C35" s="42" t="n"/>
+      <c r="D35" s="42" t="n"/>
+      <c r="E35" s="44" t="n"/>
+      <c r="F35" s="45" t="n"/>
+      <c r="G35" s="46" t="n"/>
+      <c r="H35" s="45" t="n"/>
+      <c r="I35" s="45" t="n"/>
+      <c r="J35" s="45" t="n"/>
+      <c r="K35" s="45" t="n"/>
+      <c r="L35" s="47" t="n"/>
+      <c r="M35" s="42" t="n"/>
+      <c r="N35" s="45" t="n"/>
+      <c r="O35" s="42" t="n"/>
+      <c r="P35" s="45" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="19">
+      <c r="A36" s="36">
         <f>IF(G36="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B36" s="20" t="n"/>
-      <c r="C36" s="19" t="n"/>
-      <c r="D36" s="19" t="n"/>
-      <c r="E36" s="21" t="n"/>
-      <c r="F36" s="22" t="n"/>
-      <c r="G36" s="23" t="n"/>
-      <c r="H36" s="22" t="n"/>
-      <c r="I36" s="22" t="n"/>
-      <c r="J36" s="22" t="n"/>
-      <c r="K36" s="22" t="n"/>
-      <c r="L36" s="24" t="n"/>
-      <c r="M36" s="19" t="n"/>
-      <c r="N36" s="22" t="n"/>
-      <c r="O36" s="19" t="n"/>
-      <c r="P36" s="22" t="n"/>
+      <c r="B36" s="37" t="n"/>
+      <c r="C36" s="36" t="n"/>
+      <c r="D36" s="36" t="n"/>
+      <c r="E36" s="38" t="n"/>
+      <c r="F36" s="39" t="n"/>
+      <c r="G36" s="40" t="n"/>
+      <c r="H36" s="39" t="n"/>
+      <c r="I36" s="39" t="n"/>
+      <c r="J36" s="39" t="n"/>
+      <c r="K36" s="39" t="n"/>
+      <c r="L36" s="41" t="n"/>
+      <c r="M36" s="36" t="n"/>
+      <c r="N36" s="39" t="n"/>
+      <c r="O36" s="36" t="n"/>
+      <c r="P36" s="39" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="25">
+      <c r="A37" s="42">
         <f>IF(G37="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B37" s="26" t="n"/>
-      <c r="C37" s="25" t="n"/>
-      <c r="D37" s="25" t="n"/>
-      <c r="E37" s="27" t="n"/>
-      <c r="F37" s="28" t="n"/>
-      <c r="G37" s="29" t="n"/>
-      <c r="H37" s="28" t="n"/>
-      <c r="I37" s="28" t="n"/>
-      <c r="J37" s="28" t="n"/>
-      <c r="K37" s="28" t="n"/>
-      <c r="L37" s="30" t="n"/>
-      <c r="M37" s="25" t="n"/>
-      <c r="N37" s="28" t="n"/>
-      <c r="O37" s="25" t="n"/>
-      <c r="P37" s="28" t="n"/>
+      <c r="B37" s="43" t="n"/>
+      <c r="C37" s="42" t="n"/>
+      <c r="D37" s="42" t="n"/>
+      <c r="E37" s="44" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="46" t="n"/>
+      <c r="H37" s="45" t="n"/>
+      <c r="I37" s="45" t="n"/>
+      <c r="J37" s="45" t="n"/>
+      <c r="K37" s="45" t="n"/>
+      <c r="L37" s="47" t="n"/>
+      <c r="M37" s="42" t="n"/>
+      <c r="N37" s="45" t="n"/>
+      <c r="O37" s="42" t="n"/>
+      <c r="P37" s="45" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="19">
+      <c r="A38" s="36">
         <f>IF(G38="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B38" s="20" t="n"/>
-      <c r="C38" s="19" t="n"/>
-      <c r="D38" s="19" t="n"/>
-      <c r="E38" s="21" t="n"/>
-      <c r="F38" s="22" t="n"/>
-      <c r="G38" s="23" t="n"/>
-      <c r="H38" s="22" t="n"/>
-      <c r="I38" s="22" t="n"/>
-      <c r="J38" s="22" t="n"/>
-      <c r="K38" s="22" t="n"/>
-      <c r="L38" s="24" t="n"/>
-      <c r="M38" s="19" t="n"/>
-      <c r="N38" s="22" t="n"/>
-      <c r="O38" s="19" t="n"/>
-      <c r="P38" s="22" t="n"/>
+      <c r="B38" s="37" t="n"/>
+      <c r="C38" s="36" t="n"/>
+      <c r="D38" s="36" t="n"/>
+      <c r="E38" s="38" t="n"/>
+      <c r="F38" s="39" t="n"/>
+      <c r="G38" s="40" t="n"/>
+      <c r="H38" s="39" t="n"/>
+      <c r="I38" s="39" t="n"/>
+      <c r="J38" s="39" t="n"/>
+      <c r="K38" s="39" t="n"/>
+      <c r="L38" s="41" t="n"/>
+      <c r="M38" s="36" t="n"/>
+      <c r="N38" s="39" t="n"/>
+      <c r="O38" s="36" t="n"/>
+      <c r="P38" s="39" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="25">
+      <c r="A39" s="42">
         <f>IF(G39="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B39" s="26" t="n"/>
-      <c r="C39" s="25" t="n"/>
-      <c r="D39" s="25" t="n"/>
-      <c r="E39" s="27" t="n"/>
-      <c r="F39" s="28" t="n"/>
-      <c r="G39" s="29" t="n"/>
-      <c r="H39" s="28" t="n"/>
-      <c r="I39" s="28" t="n"/>
-      <c r="J39" s="28" t="n"/>
-      <c r="K39" s="28" t="n"/>
-      <c r="L39" s="30" t="n"/>
-      <c r="M39" s="25" t="n"/>
-      <c r="N39" s="28" t="n"/>
-      <c r="O39" s="25" t="n"/>
-      <c r="P39" s="28" t="n"/>
+      <c r="B39" s="43" t="n"/>
+      <c r="C39" s="42" t="n"/>
+      <c r="D39" s="42" t="n"/>
+      <c r="E39" s="44" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="46" t="n"/>
+      <c r="H39" s="45" t="n"/>
+      <c r="I39" s="45" t="n"/>
+      <c r="J39" s="45" t="n"/>
+      <c r="K39" s="45" t="n"/>
+      <c r="L39" s="47" t="n"/>
+      <c r="M39" s="42" t="n"/>
+      <c r="N39" s="45" t="n"/>
+      <c r="O39" s="42" t="n"/>
+      <c r="P39" s="45" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="19">
+      <c r="A40" s="36">
         <f>IF(G40="","",ROW()-15)</f>
         <v/>
       </c>
-      <c r="B40" s="20" t="n"/>
-      <c r="C40" s="19" t="n"/>
-      <c r="D40" s="19" t="n"/>
-      <c r="E40" s="21" t="n"/>
-      <c r="F40" s="22" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="22" t="n"/>
-      <c r="I40" s="22" t="n"/>
-      <c r="J40" s="22" t="n"/>
-      <c r="K40" s="22" t="n"/>
-      <c r="L40" s="24" t="n"/>
-      <c r="M40" s="19" t="n"/>
-      <c r="N40" s="22" t="n"/>
-      <c r="O40" s="19" t="n"/>
-      <c r="P40" s="22" t="n"/>
+      <c r="B40" s="37" t="n"/>
+      <c r="C40" s="36" t="n"/>
+      <c r="D40" s="36" t="n"/>
+      <c r="E40" s="38" t="n"/>
+      <c r="F40" s="39" t="n"/>
+      <c r="G40" s="40" t="n"/>
+      <c r="H40" s="39" t="n"/>
+      <c r="I40" s="39" t="n"/>
+      <c r="J40" s="39" t="n"/>
+      <c r="K40" s="39" t="n"/>
+      <c r="L40" s="41" t="n"/>
+      <c r="M40" s="36" t="n"/>
+      <c r="N40" s="39" t="n"/>
+      <c r="O40" s="36" t="n"/>
+      <c r="P40" s="39" t="n"/>
     </row>
     <row r="41">
-      <c r="K41" s="31" t="inlineStr">
+      <c r="K41" s="48" t="inlineStr">
         <is>
           <t>Total pub du mois</t>
         </is>
       </c>
-      <c r="L41" s="32">
+      <c r="L41" s="49">
         <f>SUM(L16:L40)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="K42" s="31" t="inlineStr">
+      <c r="K42" s="48" t="inlineStr">
         <is>
           <t>Posts publiés</t>
         </is>
       </c>
-      <c r="L42" s="33">
+      <c r="L42" s="50">
         <f>COUNTIF(M16:M40,"Publié")&amp;" / "&amp;COUNTA(G16:G40)</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="34" t="inlineStr">
+      <c r="A44" s="21" t="inlineStr">
         <is>
           <t>Pub du mois : 300 (événement L'Annexe) + 100 (événement partenaire) + 300 (pub continue sur les meilleurs posts PRODUITS / TREND) + 1'500 (campagne fin d'année, couvre novembre et décembre).</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="34" t="inlineStr">
+      <c r="A45" s="21" t="inlineStr">
         <is>
           <t>À valider : dates et thèmes des événements [entre crochets] · contenus PRODUITS par la conformité (plafonds 3a, pas de promesse de rendement) · sons tendance à choisir la veille parmi les sons libres de droits pour compte pro.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="34" t="inlineStr">
+      <c r="A46" s="21" t="inlineStr">
         <is>
           <t>Le récap de l'événement L'Annexe se fait en stories (pas de post supplémentaire), pour garder le rythme de 2 posts par semaine.</t>
         </is>

</xml_diff>

<commit_message>
Calendrier novembre : publications mardi et vendredi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011boZbkbrQUBfZ2CayJHvQc
</commit_message>
<xml_diff>
--- a/livrables/calendrier-editorial-novembre-2026.xlsx
+++ b/livrables/calendrier-editorial-novembre-2026.xlsx
@@ -802,7 +802,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Calendrier éditorial Instagram · L'Annexe by RG · 2 posts par semaine (mardi et jeudi, 12h15) · 2 EVENT par mois (L'Annexe + partenaire), le reste en PRODUITS et TREND</t>
+          <t>Calendrier éditorial Instagram · L'Annexe by RG · 2 posts par semaine (mardi et vendredi, 12h15) · 2 EVENT par mois (L'Annexe + partenaire), le reste en PRODUITS et TREND</t>
         </is>
       </c>
     </row>
@@ -920,13 +920,13 @@
       <c r="C8" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>5   ·   EVENT</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="n">
-        <v>6</v>
+      <c r="D8" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>6   ·   EVENT</t>
+        </is>
       </c>
       <c r="F8" s="10" t="n">
         <v>7</v>
@@ -949,14 +949,14 @@
           <t>Story · Quiz du mercredi</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>Post
 Événement L'Annexe · [titre de l'événement de novembre]
 12h15  ·  pub 300 CHF</t>
         </is>
       </c>
-      <c r="E9" s="15" t="n"/>
       <c r="F9" s="11" t="n"/>
       <c r="G9" s="11" t="n"/>
     </row>
@@ -972,13 +972,13 @@
       <c r="C10" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>12   ·   PRODUITS</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="n">
-        <v>13</v>
+      <c r="D10" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>13   ·   PRODUITS</t>
+        </is>
       </c>
       <c r="F10" s="10" t="n">
         <v>14</v>
@@ -1001,14 +1001,14 @@
           <t>Story · Quiz du mercredi</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>Reel
 Combien tu économiserais d'impôts avec ton 3a ? On fait le test.
 12h15  ·  pub 150 CHF</t>
         </is>
       </c>
-      <c r="E11" s="15" t="n"/>
       <c r="F11" s="11" t="n"/>
       <c r="G11" s="11" t="n"/>
     </row>
@@ -1024,13 +1024,13 @@
       <c r="C12" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>19   ·   TREND</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="n">
-        <v>20</v>
+      <c r="D12" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>20   ·   TREND</t>
+        </is>
       </c>
       <c r="F12" s="10" t="n">
         <v>21</v>
@@ -1053,14 +1053,14 @@
           <t>Story · Quiz du mercredi</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="20" t="inlineStr">
         <is>
           <t>Reel
 Ce que j'aurais aimé savoir sur l'argent à 25 ans
 12h15  ·  pub 150 CHF</t>
         </is>
       </c>
-      <c r="E13" s="15" t="n"/>
       <c r="F13" s="11" t="n"/>
       <c r="G13" s="11" t="n"/>
     </row>
@@ -1076,13 +1076,13 @@
       <c r="C14" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>26   ·   TREND</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>27</v>
+      <c r="D14" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>27   ·   TREND</t>
+        </is>
       </c>
       <c r="F14" s="10" t="n">
         <v>28</v>
@@ -1105,14 +1105,14 @@
           <t>Story · Quiz du mercredi</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="20" t="inlineStr">
         <is>
           <t>Reel
 Dis-moi que tu es freelance sans me dire que tu es freelance
 12h15</t>
         </is>
       </c>
-      <c r="E15" s="15" t="n"/>
       <c r="F15" s="11" t="n"/>
       <c r="G15" s="11" t="n"/>
     </row>
@@ -1205,7 +1205,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Règle : 2 posts par semaine (mardi et jeudi, 12h15), piliers en alternance · chaque mois : 2 EVENT (1 événement L'Annexe + 1 événement partenaire), le reste en PRODUITS et TREND · Fil rouge de novembre : versement 3a avant le 31.12</t>
+          <t>Règle : 2 posts par semaine (mardi et vendredi, 12h15), piliers en alternance · chaque mois : 2 EVENT (1 événement L'Annexe + 1 événement partenaire), le reste en PRODUITS et TREND · Fil rouge de novembre : versement 3a avant le 31.12</t>
         </is>
       </c>
     </row>
@@ -1267,7 +1267,7 @@
       <c r="F7" s="27" t="n"/>
       <c r="G7" s="26" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="H7" s="27" t="n"/>
@@ -1293,7 +1293,7 @@
       <c r="F8" s="30" t="n"/>
       <c r="G8" s="31" t="inlineStr">
         <is>
-          <t>05.11 · EVENT · Post
+          <t>06.11 · EVENT · Post
 Événement L'Annexe · [titre de l'événement de novembre]</t>
         </is>
       </c>
@@ -1320,7 +1320,7 @@
       <c r="F9" s="34" t="n"/>
       <c r="G9" s="29" t="inlineStr">
         <is>
-          <t>12.11 · PRODUITS · Reel
+          <t>13.11 · PRODUITS · Reel
 Combien tu économiserais d'impôts avec ton 3a ? On fait le test.</t>
         </is>
       </c>
@@ -1347,7 +1347,7 @@
       <c r="F10" s="32" t="n"/>
       <c r="G10" s="33" t="inlineStr">
         <is>
-          <t>19.11 · TREND · Reel
+          <t>20.11 · TREND · Reel
 Ce que j'aurais aimé savoir sur l'argent à 25 ans</t>
         </is>
       </c>
@@ -1374,7 +1374,7 @@
       <c r="F11" s="30" t="n"/>
       <c r="G11" s="33" t="inlineStr">
         <is>
-          <t>26.11 · TREND · Reel
+          <t>27.11 · TREND · Reel
 Dis-moi que tu es freelance sans me dire que tu es freelance</t>
         </is>
       </c>
@@ -1548,11 +1548,11 @@
         <v/>
       </c>
       <c r="B17" s="43" t="n">
-        <v>46331</v>
+        <v>46332</v>
       </c>
       <c r="C17" s="42" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="D17" s="42" t="inlineStr">
@@ -1686,11 +1686,11 @@
         <v/>
       </c>
       <c r="B19" s="43" t="n">
-        <v>46338</v>
+        <v>46339</v>
       </c>
       <c r="C19" s="42" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="D19" s="42" t="inlineStr">
@@ -1824,11 +1824,11 @@
         <v/>
       </c>
       <c r="B21" s="43" t="n">
-        <v>46345</v>
+        <v>46346</v>
       </c>
       <c r="C21" s="42" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="D21" s="42" t="inlineStr">
@@ -1962,11 +1962,11 @@
         <v/>
       </c>
       <c r="B23" s="43" t="n">
-        <v>46352</v>
+        <v>46353</v>
       </c>
       <c r="C23" s="42" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="D23" s="42" t="inlineStr">

</xml_diff>